<commit_message>
Minimum Viable Product (MVP)
</commit_message>
<xml_diff>
--- a/sinif_listesi/ogrenciler.xlsx
+++ b/sinif_listesi/ogrenciler.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Isim</t>
+          <t>Ad_Soyad</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -434,19 +434,27 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>245541023</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>245541023</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>memet</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>monur boyraz</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>204420102</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>204420102</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -456,8 +464,10 @@
       <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>123456789</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>123456789</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -467,8 +477,10 @@
       <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>987654321</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>987654321</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -478,8 +490,10 @@
       <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>111222333</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>111222333</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -489,8 +503,10 @@
       <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>456789123</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>456789123</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>

</xml_diff>